<commit_message>
data: publish 2026-09-07 daily operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-07-上海公交运营.xlsx
+++ b/data/export/2026-09-07-上海公交运营.xlsx
@@ -13,8 +13,8 @@
     <sheet name="182路" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'全部班次'!$A$1:$S$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'浦东78路'!$A$1:$S$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'全部班次'!$A$1:$S$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'浦东78路'!$A$1:$S$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'浦东35路'!$A$1:$S$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'182路'!$A$1:$S$4</definedName>
   </definedNames>
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S8"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -429,17 +429,17 @@
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="6" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
     <col width="8" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
@@ -570,10 +570,14 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>22:22</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -586,17 +590,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点近站ETA</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -606,12 +610,20 @@
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
       <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S2" t="n">
+        <v>67</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -641,10 +653,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -657,17 +673,17 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点近站ETA</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -677,12 +693,20 @@
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>2</v>
+      </c>
       <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S3" t="n">
+        <v>68</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -712,10 +736,14 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>21:41</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -728,17 +756,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>末次终点ETA</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -748,12 +776,20 @@
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>末次终点ETA推算，约±15分钟</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>3</v>
+      </c>
       <c r="R4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S4" t="n">
+        <v>71</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -783,10 +819,14 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>22:46</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -799,17 +839,17 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点近站ETA</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -819,12 +859,20 @@
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±2分钟</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>1</v>
+      </c>
       <c r="R5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S5" t="n">
+        <v>111</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -854,10 +902,14 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>22:46</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -870,17 +922,17 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点近站ETA</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -890,12 +942,20 @@
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±2分钟</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>2</v>
+      </c>
       <c r="R6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S6" t="n">
+        <v>136</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -925,10 +985,14 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>21:54</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -941,17 +1005,17 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>末次终点ETA</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -961,12 +1025,20 @@
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>末次终点ETA推算，约±10分钟</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>3</v>
+      </c>
       <c r="R7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S7" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -996,10 +1068,14 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>22:21</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1012,17 +1088,17 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点近站ETA</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1032,15 +1108,106 @@
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>2</v>
+      </c>
       <c r="R8" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S8" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>浦东78路</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>沪A56630D</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>SHMAAS待发计划</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>未发现可靠中途折返证据</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>终点近站ETA</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±2分钟</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>1</v>
+      </c>
+      <c r="R9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" t="n">
+        <v>65</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S8"/>
+  <autoFilter ref="A1:S9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1051,7 +1218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1059,17 +1226,17 @@
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="6" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
     <col width="8" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
@@ -1200,10 +1367,14 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>21:54</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1216,17 +1387,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>末次终点ETA</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -1236,12 +1407,20 @@
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>末次终点ETA推算，约±10分钟</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>3</v>
+      </c>
       <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S2" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1271,10 +1450,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>22:21</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1287,17 +1470,17 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点近站ETA</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -1307,15 +1490,106 @@
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>2</v>
+      </c>
       <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S3" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>浦东78路</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>沪A56630D</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SHMAAS待发计划</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>未发现可靠中途折返证据</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>终点近站ETA</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±2分钟</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" t="n">
+        <v>65</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S3"/>
+  <autoFilter ref="A1:S4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1334,17 +1608,17 @@
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="6" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
     <col width="8" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
@@ -1475,10 +1749,14 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>22:46</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1491,17 +1769,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点近站ETA</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -1511,12 +1789,20 @@
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±2分钟</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
       <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S2" t="n">
+        <v>111</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1546,10 +1832,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>22:46</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1562,17 +1852,17 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点近站ETA</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -1582,12 +1872,20 @@
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±2分钟</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>2</v>
+      </c>
       <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S3" t="n">
+        <v>136</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S3"/>
@@ -1609,17 +1907,17 @@
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="6" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="4" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
     <col width="8" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
@@ -1750,10 +2048,14 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>22:22</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1766,17 +2068,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点近站ETA</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -1786,12 +2088,20 @@
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
       <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S2" t="n">
+        <v>67</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1821,10 +2131,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1837,17 +2151,17 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>终点近站ETA</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -1857,12 +2171,20 @@
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>终点近站ETA推算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>2</v>
+      </c>
       <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S3" t="n">
+        <v>68</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1892,10 +2214,14 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>21:41</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1908,17 +2234,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>末次终点ETA</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -1928,12 +2254,20 @@
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>末次终点ETA推算，约±15分钟</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>3</v>
+      </c>
       <c r="R4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S4" t="n">
+        <v>71</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:S4"/>

</xml_diff>